<commit_message>
M2 complete: Locked verified reference map for BTM-CH01
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -10,7 +10,7 @@
     <sheet name="chiller_products_draft" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">chiller_products_draft!$D$1:$D$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">chiller_products_draft!$D$1:$D$51</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="210">
   <si>
     <t>product_id</t>
   </si>
@@ -71,7 +71,7 @@
     <t>image_url</t>
   </si>
   <si>
-    <t>RASKIK_150</t>
+    <t>RASKIK_MANGO_150</t>
   </si>
   <si>
     <t>Raskik 150ml mango</t>
@@ -278,6 +278,18 @@
     <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304179511_IMG1V2.webp</t>
   </si>
   <si>
+    <t>THUMSUP_XFORCE_300</t>
+  </si>
+  <si>
+    <t>Thums up xforce 300ml</t>
+  </si>
+  <si>
+    <t>Thums Up</t>
+  </si>
+  <si>
+    <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304191882_PL0AFRO1.webp</t>
+  </si>
+  <si>
     <t>DIET_COKE_300</t>
   </si>
   <si>
@@ -365,9 +377,6 @@
     <t>Thums Up 250ml</t>
   </si>
   <si>
-    <t>Thums Up</t>
-  </si>
-  <si>
     <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304369600_PL0AFRO3.webp</t>
   </si>
   <si>
@@ -383,6 +392,15 @@
     <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304484780_PL0AFRO1.webp</t>
   </si>
   <si>
+    <t>COCACOLA_ZERO_300</t>
+  </si>
+  <si>
+    <t>Coca-Cola Coke, 330ml Can</t>
+  </si>
+  <si>
+    <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304368671_PL0AFRO1.webp</t>
+  </si>
+  <si>
     <t>AMUL_PREMIUM_BUTTERMILK_200</t>
   </si>
   <si>
@@ -410,6 +428,15 @@
     <t>https://www.bigbasket.com/pd/40256631/nandini-goodlife-pista-flavoured-milk-nutritious-healthy-classic-taste-200-ml/</t>
   </si>
   <si>
+    <t>NANDINI_CHOCOLATE_MILKSHAKE_180</t>
+  </si>
+  <si>
+    <t>Nandini Good Life Chocolate Milkshake, 180ml Bottle</t>
+  </si>
+  <si>
+    <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304539691_PL0AFRO1.webp</t>
+  </si>
+  <si>
     <t>NANDINI_MANGO_LASSI_180</t>
   </si>
   <si>
@@ -491,13 +518,10 @@
     <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304601898_PL0AFRO2.webp</t>
   </si>
   <si>
-    <t>RASKIN_NIMBU_PANI_160</t>
-  </si>
-  <si>
-    <t>Raskin Nimbu Pani 160ml</t>
-  </si>
-  <si>
-    <t>Raskin</t>
+    <t>RASKIK_NIMBU_PANI_160</t>
+  </si>
+  <si>
+    <t>Raskik Nimbu Pani 160ml</t>
   </si>
   <si>
     <t>FROOTI_200</t>
@@ -527,6 +551,18 @@
     <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304190712_PL0AFRO1.webp</t>
   </si>
   <si>
+    <t>DAILEE_MANGO_180</t>
+  </si>
+  <si>
+    <t>Dailee Enrich Alphonso Fruit Drink, Mango, 180ml Bottle</t>
+  </si>
+  <si>
+    <t>Dailee</t>
+  </si>
+  <si>
+    <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304566710_PL0AFRO1.webp</t>
+  </si>
+  <si>
     <t>CAMPA_COLA_250</t>
   </si>
   <si>
@@ -590,7 +626,7 @@
     <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304468454_PL0AFRO1.webp</t>
   </si>
   <si>
-    <t>TATA_COPPER_PLUS_1L</t>
+    <t>TATA_COPPER_PLUS_1000</t>
   </si>
   <si>
     <t>Tata Copper Plus Mineral Water 1L</t>
@@ -603,6 +639,27 @@
   </si>
   <si>
     <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304597621_PL0AFRO1.webp</t>
+  </si>
+  <si>
+    <t>SLICE_MANGO_1250</t>
+  </si>
+  <si>
+    <t>Slice Mango Drink, 1.2L Bottle</t>
+  </si>
+  <si>
+    <t>Slice</t>
+  </si>
+  <si>
+    <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304469702_PL0AFRO1.webp</t>
+  </si>
+  <si>
+    <t>BISLERI_WATER_1000</t>
+  </si>
+  <si>
+    <t>Bisleri Mineral Water, 1L Bottle</t>
+  </si>
+  <si>
+    <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304478845_PL0AFRO12.webp</t>
   </si>
 </sst>
 </file>
@@ -615,7 +672,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -650,6 +707,19 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <charset val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1115,129 +1185,132 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1"/>
@@ -1248,13 +1321,21 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1788,10 +1869,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr defaultColWidth="10.2857142857143" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="47.2857142857143" customWidth="1"/>
+    <col min="1" max="1" width="47.2857142857143" style="1" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
     <col min="3" max="3" width="13.1428571428571" customWidth="1"/>
     <col min="4" max="4" width="19.5714285714286" customWidth="1"/>
@@ -1806,7 +1887,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -1847,7 +1928,7 @@
       </c>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B2" t="s">
@@ -1871,18 +1952,21 @@
       <c r="H2" t="s">
         <v>18</v>
       </c>
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
       <c r="K2" t="b">
         <v>0</v>
       </c>
       <c r="L2" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="M2" s="2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B3" t="s">
@@ -1906,18 +1990,21 @@
       <c r="H3" t="s">
         <v>18</v>
       </c>
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
       <c r="K3" t="b">
         <v>0</v>
       </c>
       <c r="L3" t="s">
         <v>19</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="M3" s="3" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B4" t="s">
@@ -1941,18 +2028,21 @@
       <c r="H4" t="s">
         <v>18</v>
       </c>
+      <c r="J4" t="b">
+        <v>0</v>
+      </c>
       <c r="K4" t="b">
         <v>0</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M4" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B5" t="s">
@@ -1976,6 +2066,9 @@
       <c r="H5" t="s">
         <v>18</v>
       </c>
+      <c r="J5" t="b">
+        <v>0</v>
+      </c>
       <c r="K5" t="b">
         <v>0</v>
       </c>
@@ -1987,7 +2080,7 @@
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B6" t="s">
@@ -2011,6 +2104,9 @@
       <c r="H6" t="s">
         <v>18</v>
       </c>
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
       <c r="K6" t="b">
         <v>0</v>
       </c>
@@ -2022,7 +2118,7 @@
       </c>
     </row>
     <row r="7" spans="1:13">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B7" t="s">
@@ -2046,6 +2142,9 @@
       <c r="H7" t="s">
         <v>18</v>
       </c>
+      <c r="J7" t="b">
+        <v>0</v>
+      </c>
       <c r="K7" t="b">
         <v>0</v>
       </c>
@@ -2057,7 +2156,7 @@
       </c>
     </row>
     <row r="8" spans="1:13">
-      <c r="A8" t="s">
+      <c r="A8" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B8" t="s">
@@ -2081,6 +2180,9 @@
       <c r="H8" t="s">
         <v>18</v>
       </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
       <c r="K8" t="b">
         <v>0</v>
       </c>
@@ -2092,7 +2194,7 @@
       </c>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B9" t="s">
@@ -2116,6 +2218,9 @@
       <c r="H9" t="s">
         <v>18</v>
       </c>
+      <c r="J9" t="b">
+        <v>0</v>
+      </c>
       <c r="K9" t="b">
         <v>0</v>
       </c>
@@ -2127,7 +2232,7 @@
       </c>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B10" t="s">
@@ -2151,6 +2256,9 @@
       <c r="H10" t="s">
         <v>18</v>
       </c>
+      <c r="J10" t="b">
+        <v>0</v>
+      </c>
       <c r="K10" t="b">
         <v>0</v>
       </c>
@@ -2162,7 +2270,7 @@
       </c>
     </row>
     <row r="11" customFormat="1" spans="1:13">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B11" t="s">
@@ -2186,6 +2294,9 @@
       <c r="H11" t="s">
         <v>18</v>
       </c>
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
       <c r="K11" t="b">
         <v>0</v>
       </c>
@@ -2197,7 +2308,7 @@
       </c>
     </row>
     <row r="12" customFormat="1" spans="1:13">
-      <c r="A12" t="s">
+      <c r="A12" s="1" t="s">
         <v>58</v>
       </c>
       <c r="B12" t="s">
@@ -2221,18 +2332,21 @@
       <c r="H12" t="s">
         <v>61</v>
       </c>
+      <c r="J12" t="b">
+        <v>0</v>
+      </c>
       <c r="K12" t="b">
         <v>0</v>
       </c>
       <c r="L12" t="s">
         <v>56</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="M12" s="5" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="13" customFormat="1" spans="1:13">
-      <c r="A13" t="s">
+      <c r="A13" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B13" t="s">
@@ -2256,6 +2370,9 @@
       <c r="H13" t="s">
         <v>61</v>
       </c>
+      <c r="J13" t="b">
+        <v>0</v>
+      </c>
       <c r="K13" t="b">
         <v>0</v>
       </c>
@@ -2267,7 +2384,7 @@
       </c>
     </row>
     <row r="14" customFormat="1" spans="1:13">
-      <c r="A14" t="s">
+      <c r="A14" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B14" t="s">
@@ -2291,6 +2408,9 @@
       <c r="H14" t="s">
         <v>18</v>
       </c>
+      <c r="J14" t="b">
+        <v>0</v>
+      </c>
       <c r="K14" t="b">
         <v>0</v>
       </c>
@@ -2302,7 +2422,7 @@
       </c>
     </row>
     <row r="15" customFormat="1" spans="1:13">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>70</v>
       </c>
       <c r="B15" t="s">
@@ -2326,6 +2446,9 @@
       <c r="H15" t="s">
         <v>18</v>
       </c>
+      <c r="J15" t="b">
+        <v>0</v>
+      </c>
       <c r="K15" t="b">
         <v>0</v>
       </c>
@@ -2337,7 +2460,7 @@
       </c>
     </row>
     <row r="16" customFormat="1" spans="1:13">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B16" t="s">
@@ -2361,6 +2484,9 @@
       <c r="H16" t="s">
         <v>18</v>
       </c>
+      <c r="J16" t="b">
+        <v>0</v>
+      </c>
       <c r="K16" t="b">
         <v>0</v>
       </c>
@@ -2372,7 +2498,7 @@
       </c>
     </row>
     <row r="17" spans="1:13">
-      <c r="A17" t="s">
+      <c r="A17" s="1" t="s">
         <v>78</v>
       </c>
       <c r="B17" t="s">
@@ -2396,6 +2522,9 @@
       <c r="H17" t="s">
         <v>18</v>
       </c>
+      <c r="J17" t="b">
+        <v>0</v>
+      </c>
       <c r="K17" t="b">
         <v>0</v>
       </c>
@@ -2407,143 +2536,152 @@
       </c>
     </row>
     <row r="18" spans="1:13">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="D18" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E18" s="5">
+      <c r="D18" t="s">
+        <v>55</v>
+      </c>
+      <c r="E18" s="7">
         <v>300</v>
       </c>
       <c r="F18">
         <v>40</v>
       </c>
-      <c r="G18" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="H18" s="5" t="s">
+      <c r="G18" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H18" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="K18" s="5" t="b">
+      <c r="J18" t="b">
+        <v>0</v>
+      </c>
+      <c r="K18" s="7" t="b">
         <v>0</v>
       </c>
       <c r="L18" t="s">
         <v>56</v>
       </c>
       <c r="M18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="19" spans="1:13">
       <c r="A19" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="E19">
-        <v>250</v>
+      <c r="D19" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E19" s="7">
+        <v>300</v>
       </c>
       <c r="F19">
-        <v>125</v>
-      </c>
-      <c r="G19" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G19" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H19" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="K19" s="5" t="b">
+      <c r="J19" t="b">
+        <v>0</v>
+      </c>
+      <c r="K19" s="7" t="b">
         <v>0</v>
       </c>
       <c r="L19" t="s">
         <v>56</v>
       </c>
       <c r="M19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:13">
-      <c r="A20" t="s">
-        <v>90</v>
+      <c r="A20" s="8" t="s">
+        <v>91</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E20" s="7">
+        <v>68</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E20">
         <v>250</v>
       </c>
-      <c r="F20" s="7">
-        <v>20</v>
+      <c r="F20">
+        <v>125</v>
       </c>
       <c r="G20" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="H20" t="s">
         <v>18</v>
       </c>
-      <c r="I20" s="7"/>
-      <c r="J20" s="7"/>
-      <c r="K20" t="b">
-        <v>0</v>
-      </c>
-      <c r="L20" s="7" t="s">
-        <v>19</v>
+      <c r="J20" t="b">
+        <v>0</v>
+      </c>
+      <c r="K20" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="L20" t="s">
+        <v>56</v>
       </c>
       <c r="M20" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="21" spans="1:13">
-      <c r="A21" t="s">
+      <c r="A21" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E21" s="7">
+      <c r="D21" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E21" s="9">
         <v>250</v>
       </c>
-      <c r="F21" s="7">
+      <c r="F21" s="9">
         <v>20</v>
       </c>
-      <c r="G21" s="7" t="s">
+      <c r="G21" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H21" s="7" t="s">
+      <c r="H21" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I21" s="7"/>
-      <c r="J21" s="7"/>
+      <c r="I21" s="9"/>
+      <c r="J21" t="b">
+        <v>0</v>
+      </c>
       <c r="K21" t="b">
         <v>0</v>
       </c>
-      <c r="L21" s="7" t="s">
+      <c r="L21" s="9" t="s">
         <v>19</v>
       </c>
       <c r="M21" t="s">
@@ -2551,36 +2689,38 @@
       </c>
     </row>
     <row r="22" spans="1:13">
-      <c r="A22" t="s">
+      <c r="A22" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="D22" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E22" s="7">
+      <c r="D22" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E22" s="9">
         <v>250</v>
       </c>
-      <c r="F22" s="7">
+      <c r="F22" s="9">
         <v>20</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="G22" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H22" s="7" t="s">
+      <c r="H22" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I22" s="7"/>
-      <c r="J22" s="7"/>
+      <c r="I22" s="9"/>
+      <c r="J22" t="b">
+        <v>0</v>
+      </c>
       <c r="K22" t="b">
         <v>0</v>
       </c>
-      <c r="L22" s="7" t="s">
+      <c r="L22" s="9" t="s">
         <v>19</v>
       </c>
       <c r="M22" t="s">
@@ -2588,36 +2728,38 @@
       </c>
     </row>
     <row r="23" spans="1:13">
-      <c r="A23" t="s">
+      <c r="A23" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="D23" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E23" s="7">
+      <c r="D23" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E23" s="9">
         <v>250</v>
       </c>
-      <c r="F23" s="7">
+      <c r="F23" s="9">
         <v>20</v>
       </c>
-      <c r="G23" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H23" s="7" t="s">
+      <c r="G23" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H23" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7"/>
+      <c r="I23" s="9"/>
+      <c r="J23" t="b">
+        <v>0</v>
+      </c>
       <c r="K23" t="b">
         <v>0</v>
       </c>
-      <c r="L23" s="7" t="s">
+      <c r="L23" s="9" t="s">
         <v>19</v>
       </c>
       <c r="M23" t="s">
@@ -2625,73 +2767,77 @@
       </c>
     </row>
     <row r="24" spans="1:13">
-      <c r="A24" t="s">
+      <c r="A24" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="C24" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E24" s="7">
+      <c r="C24" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E24" s="9">
         <v>250</v>
       </c>
-      <c r="F24" s="7">
+      <c r="F24" s="9">
         <v>20</v>
       </c>
-      <c r="G24" s="7" t="s">
+      <c r="G24" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="H24" s="7" t="s">
+      <c r="H24" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I24" s="7"/>
-      <c r="J24" s="7"/>
+      <c r="I24" s="9"/>
+      <c r="J24" t="b">
+        <v>0</v>
+      </c>
       <c r="K24" t="b">
         <v>0</v>
       </c>
-      <c r="L24" s="7" t="s">
+      <c r="L24" s="9" t="s">
         <v>19</v>
       </c>
       <c r="M24" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="25" spans="1:13">
-      <c r="A25" t="s">
-        <v>109</v>
-      </c>
-      <c r="B25" s="7" t="s">
+      <c r="A25" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="B25" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="D25" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E25" s="7">
+      <c r="C25" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E25" s="9">
         <v>250</v>
       </c>
-      <c r="F25" s="7">
+      <c r="F25" s="9">
         <v>20</v>
       </c>
-      <c r="G25" s="7" t="s">
+      <c r="G25" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="H25" s="7" t="s">
+      <c r="H25" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I25" s="7"/>
-      <c r="J25" s="7"/>
+      <c r="I25" s="9"/>
+      <c r="J25" t="b">
+        <v>0</v>
+      </c>
       <c r="K25" t="b">
         <v>0</v>
       </c>
-      <c r="L25" s="7" t="s">
+      <c r="L25" s="9" t="s">
         <v>19</v>
       </c>
       <c r="M25" t="s">
@@ -2699,184 +2845,194 @@
       </c>
     </row>
     <row r="26" spans="1:13">
-      <c r="A26" t="s">
+      <c r="A26" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E26" s="9">
+        <v>250</v>
+      </c>
+      <c r="F26" s="9">
+        <v>20</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I26" s="9"/>
+      <c r="J26" t="b">
+        <v>0</v>
+      </c>
+      <c r="K26" t="b">
+        <v>0</v>
+      </c>
+      <c r="L26" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M26" t="s">
         <v>115</v>
       </c>
-      <c r="D26" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E26" s="7">
+    </row>
+    <row r="27" spans="1:13">
+      <c r="A27" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E27" s="9">
         <v>250</v>
       </c>
-      <c r="F26" s="7">
+      <c r="F27" s="9">
         <v>20</v>
       </c>
-      <c r="G26" s="7" t="s">
+      <c r="G27" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H26" s="7" t="s">
+      <c r="H27" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7"/>
-      <c r="K26" t="b">
-        <v>0</v>
-      </c>
-      <c r="L26" s="7" t="s">
+      <c r="I27" s="9"/>
+      <c r="J27" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K27" t="b">
+        <v>0</v>
+      </c>
+      <c r="L27" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="M26" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13">
-      <c r="A27" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="C27" s="7" t="s">
+      <c r="M27" t="s">
         <v>119</v>
       </c>
-      <c r="D27" s="7" t="s">
+    </row>
+    <row r="28" spans="1:13">
+      <c r="A28" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="E27" s="7">
+      <c r="B28" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E28" s="9">
+        <v>300</v>
+      </c>
+      <c r="F28" s="9">
+        <v>40</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I28" s="9"/>
+      <c r="J28" t="b">
+        <v>0</v>
+      </c>
+      <c r="K28" t="b">
+        <v>0</v>
+      </c>
+      <c r="L28" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="M28" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
+      <c r="A29" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="E29" s="9">
         <v>200</v>
       </c>
-      <c r="F27" s="7">
+      <c r="F29" s="9">
         <v>10</v>
       </c>
-      <c r="G27" s="7" t="s">
+      <c r="G29" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H27" s="7" t="s">
+      <c r="H29" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I27" s="7"/>
-      <c r="J27" s="7"/>
-      <c r="K27" t="b">
-        <v>0</v>
-      </c>
-      <c r="L27" s="7" t="s">
+      <c r="I29" s="9"/>
+      <c r="J29" t="b">
+        <v>0</v>
+      </c>
+      <c r="K29" t="b">
+        <v>0</v>
+      </c>
+      <c r="L29" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M27" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13">
-      <c r="A28" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="E28" s="7">
+      <c r="M29" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
+      <c r="A30" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="E30" s="9">
         <v>180</v>
       </c>
-      <c r="F28" s="7">
+      <c r="F30" s="9">
         <v>25</v>
       </c>
-      <c r="G28" s="7" t="s">
+      <c r="G30" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H28" s="7" t="s">
+      <c r="H30" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I28" s="7"/>
-      <c r="J28" s="7"/>
-      <c r="K28" t="b">
-        <v>0</v>
-      </c>
-      <c r="L28" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="M28" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13">
-      <c r="A29" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="E29" s="7">
-        <v>180</v>
-      </c>
-      <c r="F29" s="7">
-        <v>25</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I29" s="7"/>
-      <c r="J29" s="7"/>
-      <c r="K29" t="b">
-        <v>0</v>
-      </c>
-      <c r="L29" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="M29" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13">
-      <c r="A30" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="D30" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="E30" s="7">
-        <v>200</v>
-      </c>
-      <c r="F30" s="7">
-        <v>25</v>
-      </c>
-      <c r="G30" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I30" s="7"/>
-      <c r="J30" s="7"/>
+      <c r="I30" s="9"/>
+      <c r="J30" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="K30" t="b">
         <v>0</v>
       </c>
-      <c r="L30" s="7" t="s">
+      <c r="L30" s="9" t="s">
         <v>19</v>
       </c>
       <c r="M30" t="s">
@@ -2884,110 +3040,116 @@
       </c>
     </row>
     <row r="31" spans="1:13">
-      <c r="A31" s="7" t="s">
+      <c r="A31" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="C31" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="E31" s="9">
+        <v>180</v>
+      </c>
+      <c r="F31" s="9">
+        <v>30</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I31" s="9"/>
+      <c r="J31" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K31" t="b">
+        <v>0</v>
+      </c>
+      <c r="L31" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M31" t="s">
         <v>134</v>
       </c>
-      <c r="D31" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="E31" s="7">
-        <v>250</v>
-      </c>
-      <c r="F31" s="7">
-        <v>120</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H31" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="I31" s="7"/>
-      <c r="J31" s="7"/>
-      <c r="K31" t="b">
-        <v>0</v>
-      </c>
-      <c r="L31" s="7" t="s">
+    </row>
+    <row r="32" spans="1:13">
+      <c r="A32" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="E32" s="9">
+        <v>180</v>
+      </c>
+      <c r="F32" s="9">
+        <v>25</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I32" s="9"/>
+      <c r="J32" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L32" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="M31" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13">
-      <c r="A32" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="B32" s="7" t="s">
+      <c r="M32" t="s">
         <v>137</v>
       </c>
-      <c r="C32" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="E32" s="7">
-        <v>250</v>
-      </c>
-      <c r="F32" s="7">
-        <v>120</v>
-      </c>
-      <c r="G32" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H32" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="I32" s="7"/>
-      <c r="J32" s="7"/>
-      <c r="K32" t="b">
-        <v>0</v>
-      </c>
-      <c r="L32" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="M32" t="s">
-        <v>135</v>
-      </c>
     </row>
     <row r="33" spans="1:13">
-      <c r="A33" s="7" t="s">
+      <c r="A33" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="C33" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="E33" s="7">
-        <v>180</v>
-      </c>
-      <c r="F33" s="7">
-        <v>20</v>
-      </c>
-      <c r="G33" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H33" s="7" t="s">
+      <c r="C33" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="E33" s="9">
+        <v>200</v>
+      </c>
+      <c r="F33" s="9">
+        <v>25</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H33" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I33" s="7"/>
-      <c r="J33" s="7"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="K33" t="b">
         <v>0</v>
       </c>
-      <c r="L33" s="7" t="s">
+      <c r="L33" s="9" t="s">
         <v>19</v>
       </c>
       <c r="M33" t="s">
@@ -2995,221 +3157,233 @@
       </c>
     </row>
     <row r="34" spans="1:13">
-      <c r="A34" s="7" t="s">
+      <c r="A34" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="C34" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D34" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E34" s="7">
-        <v>200</v>
-      </c>
-      <c r="F34" s="7">
-        <v>10</v>
-      </c>
-      <c r="G34" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H34" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I34" s="7"/>
-      <c r="J34" s="7"/>
+      <c r="C34" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="E34" s="9">
+        <v>250</v>
+      </c>
+      <c r="F34" s="9">
+        <v>120</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H34" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="K34" t="b">
         <v>0</v>
       </c>
-      <c r="L34" s="7" t="s">
-        <v>143</v>
+      <c r="L34" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="M34" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="35" spans="1:13">
-      <c r="A35" s="7" t="s">
+      <c r="A35" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B35" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="C35" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="E35" s="9">
+        <v>250</v>
+      </c>
+      <c r="F35" s="9">
+        <v>120</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H35" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K35" t="b">
+        <v>0</v>
+      </c>
+      <c r="L35" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M35" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13">
+      <c r="A36" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="B36" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="E36" s="9">
+        <v>180</v>
+      </c>
+      <c r="F36" s="9">
+        <v>20</v>
+      </c>
+      <c r="G36" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H36" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I36" s="9"/>
+      <c r="J36" t="b">
+        <v>0</v>
+      </c>
+      <c r="K36" t="b">
+        <v>0</v>
+      </c>
+      <c r="L36" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M36" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13">
+      <c r="A37" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D37" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E35" s="7">
+      <c r="E37" s="9">
         <v>200</v>
       </c>
-      <c r="F35" s="7">
+      <c r="F37" s="9">
+        <v>10</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H37" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I37" s="9"/>
+      <c r="J37" t="b">
+        <v>0</v>
+      </c>
+      <c r="K37" t="b">
+        <v>0</v>
+      </c>
+      <c r="L37" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="M37" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13">
+      <c r="A38" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E38" s="9">
+        <v>200</v>
+      </c>
+      <c r="F38" s="9">
         <v>20</v>
       </c>
-      <c r="G35" s="7" t="s">
+      <c r="G38" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H35" s="7" t="s">
+      <c r="H38" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I35" s="7"/>
-      <c r="J35" s="7"/>
-      <c r="K35" t="b">
-        <v>0</v>
-      </c>
-      <c r="L35" s="7" t="s">
+      <c r="I38" s="9"/>
+      <c r="J38" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K38" t="b">
+        <v>0</v>
+      </c>
+      <c r="L38" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="M35" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13">
-      <c r="A36" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="B36" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="D36" s="7" t="s">
+      <c r="M38" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13">
+      <c r="A39" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="D39" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E36" s="7">
+      <c r="E39" s="9">
         <v>160</v>
       </c>
-      <c r="F36" s="7">
+      <c r="F39" s="9">
         <v>10</v>
       </c>
-      <c r="G36" s="7" t="s">
+      <c r="G39" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H36" s="7" t="s">
+      <c r="H39" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I36" s="7"/>
-      <c r="J36" s="7"/>
-      <c r="K36" t="b">
-        <v>0</v>
-      </c>
-      <c r="L36" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="M36" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13">
-      <c r="A37" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="B37" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E37" s="7">
-        <v>160</v>
-      </c>
-      <c r="F37" s="7">
-        <v>10</v>
-      </c>
-      <c r="G37" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H37" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I37" s="7"/>
-      <c r="J37" s="7"/>
-      <c r="K37" t="b">
-        <v>0</v>
-      </c>
-      <c r="L37" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="M37" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13">
-      <c r="A38" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="B38" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D38" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E38" s="7">
-        <v>200</v>
-      </c>
-      <c r="F38" s="7">
-        <v>10</v>
-      </c>
-      <c r="G38" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H38" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I38" s="7"/>
-      <c r="J38" s="7"/>
-      <c r="K38" t="b">
-        <v>0</v>
-      </c>
-      <c r="L38" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="M38" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13">
-      <c r="A39" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="B39" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E39" s="7">
-        <v>250</v>
-      </c>
-      <c r="F39" s="7">
-        <v>10</v>
-      </c>
-      <c r="G39" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H39" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I39" s="7"/>
-      <c r="J39" s="7"/>
+      <c r="I39" s="9"/>
+      <c r="J39" t="b">
+        <v>0</v>
+      </c>
       <c r="K39" t="b">
         <v>0</v>
       </c>
-      <c r="L39" s="7" t="s">
+      <c r="L39" s="9" t="s">
         <v>19</v>
       </c>
       <c r="M39" t="s">
@@ -3217,293 +3391,541 @@
       </c>
     </row>
     <row r="40" spans="1:13">
-      <c r="A40" s="7" t="s">
+      <c r="A40" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="C40" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E40" s="9">
+        <v>160</v>
+      </c>
+      <c r="F40" s="9">
+        <v>10</v>
+      </c>
+      <c r="G40" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H40" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I40" s="9"/>
+      <c r="J40" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K40" t="b">
+        <v>0</v>
+      </c>
+      <c r="L40" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M40" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13">
+      <c r="A41" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E41" s="9">
+        <v>200</v>
+      </c>
+      <c r="F41" s="9">
+        <v>10</v>
+      </c>
+      <c r="G41" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H41" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I41" s="9"/>
+      <c r="J41" t="b">
+        <v>0</v>
+      </c>
+      <c r="K41" t="b">
+        <v>0</v>
+      </c>
+      <c r="L41" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M41" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13">
+      <c r="A42" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E42" s="9">
+        <v>250</v>
+      </c>
+      <c r="F42" s="9">
+        <v>10</v>
+      </c>
+      <c r="G42" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H42" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I42" s="9"/>
+      <c r="J42" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K42" t="b">
+        <v>0</v>
+      </c>
+      <c r="L42" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M42" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13">
+      <c r="A43" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="C43" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="D40" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E40" s="7">
+      <c r="D43" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="E43" s="9">
         <v>250</v>
       </c>
-      <c r="F40" s="7">
+      <c r="F43" s="9">
+        <v>10</v>
+      </c>
+      <c r="G43" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H43" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I43" s="9"/>
+      <c r="J43" t="b">
+        <v>0</v>
+      </c>
+      <c r="K43" t="b">
+        <v>0</v>
+      </c>
+      <c r="L43" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M43" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13">
+      <c r="A44" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="B44" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E44" s="9">
+        <v>180</v>
+      </c>
+      <c r="F44" s="9">
+        <v>12</v>
+      </c>
+      <c r="G44" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H44" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I44" s="9"/>
+      <c r="J44" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K44" t="b">
+        <v>0</v>
+      </c>
+      <c r="L44" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M44" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13">
+      <c r="A45" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="E45" s="9">
+        <v>250</v>
+      </c>
+      <c r="F45" s="9">
         <v>20</v>
       </c>
-      <c r="G40" s="7" t="s">
+      <c r="G45" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="H40" s="7" t="s">
+      <c r="H45" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I40" s="7"/>
-      <c r="J40" s="7"/>
-      <c r="K40" t="b">
-        <v>0</v>
-      </c>
-      <c r="L40" s="7" t="s">
+      <c r="I45" s="9"/>
+      <c r="J45" t="b">
+        <v>0</v>
+      </c>
+      <c r="K45" t="b">
+        <v>0</v>
+      </c>
+      <c r="L45" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="M40" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13">
-      <c r="A41" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="B41" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="C41" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="E41" s="7">
-        <v>250</v>
-      </c>
-      <c r="F41" s="7">
+      <c r="M45" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13">
+      <c r="A46" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="E46" s="9">
+        <v>1250</v>
+      </c>
+      <c r="F46" s="9"/>
+      <c r="G46" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H46" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="I46" s="9"/>
+      <c r="J46" t="b">
+        <v>0</v>
+      </c>
+      <c r="K46" t="b">
+        <v>0</v>
+      </c>
+      <c r="L46" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M46" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13">
+      <c r="A47" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="E47" s="9">
+        <v>1250</v>
+      </c>
+      <c r="F47" s="9"/>
+      <c r="G47" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H47" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="I47" s="9"/>
+      <c r="J47" t="b">
+        <v>0</v>
+      </c>
+      <c r="K47" t="b">
+        <v>0</v>
+      </c>
+      <c r="L47" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M47" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13">
+      <c r="A48" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="B48" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="E48" s="9">
+        <v>1250</v>
+      </c>
+      <c r="F48" s="9"/>
+      <c r="G48" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H48" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="I48" s="9"/>
+      <c r="J48" t="b">
+        <v>0</v>
+      </c>
+      <c r="K48" t="b">
+        <v>0</v>
+      </c>
+      <c r="L48" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M48" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13">
+      <c r="A49" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="E49" s="9">
+        <v>1250</v>
+      </c>
+      <c r="F49" s="9">
+        <v>60</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H49" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="I49" s="9"/>
+      <c r="J49" t="b">
+        <v>0</v>
+      </c>
+      <c r="K49" t="b">
+        <v>0</v>
+      </c>
+      <c r="L49" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M49" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13">
+      <c r="A50" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="E50" s="9">
+        <v>1250</v>
+      </c>
+      <c r="F50" s="9"/>
+      <c r="G50" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H50" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="I50" s="9"/>
+      <c r="J50" t="b">
+        <v>0</v>
+      </c>
+      <c r="K50" t="b">
+        <v>0</v>
+      </c>
+      <c r="L50" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M50" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13">
+      <c r="A51" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="E51" s="9">
+        <v>1000</v>
+      </c>
+      <c r="F51" s="9"/>
+      <c r="G51" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H51" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="I51" s="9"/>
+      <c r="J51" t="b">
+        <v>0</v>
+      </c>
+      <c r="K51" t="b">
+        <v>1</v>
+      </c>
+      <c r="L51" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M51" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13">
+      <c r="A52" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="B52" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="C52" t="s">
+        <v>205</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E52">
+        <v>1250</v>
+      </c>
+      <c r="F52">
+        <v>70</v>
+      </c>
+      <c r="G52" t="s">
+        <v>17</v>
+      </c>
+      <c r="H52" t="s">
+        <v>183</v>
+      </c>
+      <c r="J52" t="b">
+        <v>0</v>
+      </c>
+      <c r="K52" t="b">
+        <v>0</v>
+      </c>
+      <c r="L52" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M52" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13">
+      <c r="A53" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B53" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="C53" t="s">
+        <v>160</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="E53">
+        <v>1000</v>
+      </c>
+      <c r="F53">
         <v>20</v>
       </c>
-      <c r="G41" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H41" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I41" s="7"/>
-      <c r="J41" s="7"/>
-      <c r="K41" t="b">
-        <v>0</v>
-      </c>
-      <c r="L41" s="7" t="s">
+      <c r="G53" t="s">
+        <v>17</v>
+      </c>
+      <c r="H53" t="s">
+        <v>183</v>
+      </c>
+      <c r="J53" t="b">
+        <v>1</v>
+      </c>
+      <c r="K53" t="b">
+        <v>1</v>
+      </c>
+      <c r="L53" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="M41" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13">
-      <c r="A42" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="B42" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="D42" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="E42" s="7">
-        <v>1250</v>
-      </c>
-      <c r="F42" s="7"/>
-      <c r="G42" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H42" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="I42" s="7"/>
-      <c r="J42" s="7"/>
-      <c r="K42" t="b">
-        <v>0</v>
-      </c>
-      <c r="L42" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="M42" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13">
-      <c r="A43" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="B43" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="C43" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="D43" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="E43" s="7">
-        <v>1250</v>
-      </c>
-      <c r="F43" s="7"/>
-      <c r="G43" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H43" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="I43" s="7"/>
-      <c r="J43" s="7"/>
-      <c r="K43" t="b">
-        <v>0</v>
-      </c>
-      <c r="L43" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="M43" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13">
-      <c r="A44" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="B44" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="C44" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="D44" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="E44" s="7">
-        <v>1250</v>
-      </c>
-      <c r="F44" s="7"/>
-      <c r="G44" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H44" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="I44" s="7"/>
-      <c r="J44" s="7"/>
-      <c r="K44" t="b">
-        <v>0</v>
-      </c>
-      <c r="L44" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="M44" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13">
-      <c r="A45" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="B45" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="C45" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="D45" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="E45" s="7">
-        <v>1250</v>
-      </c>
-      <c r="F45" s="7">
-        <v>60</v>
-      </c>
-      <c r="G45" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H45" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="I45" s="7"/>
-      <c r="J45" s="7"/>
-      <c r="K45" t="b">
-        <v>0</v>
-      </c>
-      <c r="L45" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="M45" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="46" spans="1:13">
-      <c r="A46" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="B46" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="C46" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D46" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="E46" s="7">
-        <v>1250</v>
-      </c>
-      <c r="F46" s="7"/>
-      <c r="G46" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H46" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="I46" s="7"/>
-      <c r="J46" s="7"/>
-      <c r="K46" t="b">
-        <v>0</v>
-      </c>
-      <c r="L46" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="M46" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="47" spans="1:13">
-      <c r="A47" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="B47" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="C47" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="D47" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="E47" s="7">
-        <v>1000</v>
-      </c>
-      <c r="F47" s="7"/>
-      <c r="G47" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H47" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="I47" s="7"/>
-      <c r="J47" s="7"/>
-      <c r="K47" t="b">
-        <v>1</v>
-      </c>
-      <c r="L47" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="M47" t="s">
-        <v>190</v>
+      <c r="M53" t="s">
+        <v>209</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="D1:D47" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="D1:D51" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <hyperlinks>

</xml_diff>

<commit_message>
Fix cropping logic for edge cases
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -10,7 +10,7 @@
     <sheet name="chiller_products_draft" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">chiller_products_draft!$D$1:$D$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">chiller_products_draft!$D$1:$D$53</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -95,7 +95,7 @@
     <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304187812_IMG1V2.webp</t>
   </si>
   <si>
-    <t>MAAZA_270</t>
+    <t>MAAZA_MANGO_270</t>
   </si>
   <si>
     <t>Maaza 270ml mango</t>
@@ -110,7 +110,7 @@
     <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304478926_PL0AFRO10.webp</t>
   </si>
   <si>
-    <t>MAAZA_150</t>
+    <t>MAAZA_MANGO_150</t>
   </si>
   <si>
     <t>Maaza 150ml mango</t>
@@ -134,7 +134,7 @@
     <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304103248_PL0AFRO1.webp</t>
   </si>
   <si>
-    <t>SWING_270</t>
+    <t>SWING_POMEGRANATE_270</t>
   </si>
   <si>
     <t>Swing pomegranate 270ml</t>
@@ -266,7 +266,7 @@
     <t>https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304469524_PL0AFRO3.webp</t>
   </si>
   <si>
-    <t>CAMPA_ENERGY_185</t>
+    <t>CAMPA_ENERGY_gold_185</t>
   </si>
   <si>
     <t>Campa Energy Gold 185ml</t>
@@ -2531,7 +2531,7 @@
       <c r="L17" t="s">
         <v>56</v>
       </c>
-      <c r="M17" t="s">
+      <c r="M17" s="4" t="s">
         <v>81</v>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       <c r="L45" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="M45" t="s">
+      <c r="M45" s="4" t="s">
         <v>179</v>
       </c>
     </row>
@@ -3925,13 +3925,15 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="D1:D51" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="D1:D53" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <hyperlinks>
     <hyperlink ref="M2" r:id="rId1" display="https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304187812_IMG1V2.webp"/>
     <hyperlink ref="M4" r:id="rId2" display="https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304364323_PL0AFRO3.webp"/>
     <hyperlink ref="M12" r:id="rId3" display="https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304467535_PL0AFRO3.webp" tooltip="https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304467535_PL0AFRO3.webp"/>
+    <hyperlink ref="M17" r:id="rId4" display="https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304179511_IMG1V2.webp"/>
+    <hyperlink ref="M45" r:id="rId5" display="https://jtctimages.s3.ap-south-1.amazonaws.com/JPIN-1304197905_PL0AFRO1.webp"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>